<commit_message>
feat: implement PDU HAL and driver layers and update test application logic
</commit_message>
<xml_diff>
--- a/dist/test_report.xlsx
+++ b/dist/test_report.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T5"/>
+  <dimension ref="A1:U2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -494,25 +494,30 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>LED 1-4 sang lan luot (xac nhan)</t>
+          <t>LED 1-4 sáng lần lượt (xác nhận)</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>Nut nhan BT1-4 (nhan tung nut)</t>
+          <t>Nút nhấn BT1-4 (nhấn từng nút)</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>RS485 gui/nhan loopback</t>
+          <t>Dip Switch 1-4 (gạt từng bit)</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
+          <t>RS485 gửi/nhận loopback</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
           <t>PASS/Tong</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Ket luan</t>
         </is>
@@ -526,12 +531,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-13 21:34:56</t>
+          <t>2026-06-15 12:08:02</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>COM11</t>
+          <t>COM31</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -601,328 +606,27 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Loi: BT1,BT2,BT3,BT4</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>11/13</t>
+          <t>Bo qua</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>LOI</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-06-13 21:35:44</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>COM11</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>115200</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>0.1.0</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>Bo qua</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>12/13</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
+          <t>13/14</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
         <is>
           <t>OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-06-13 22:06:54</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>COM11</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>115200</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>0.1.0</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>Loi: BT1,BT2,BT3,BT4</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>Bo qua</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>11/13</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>LOI</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-06-14 11:20:18</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>COM12</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>115200</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>0.1.0</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>Loi: BT1,BT2,BT3,BT4</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>Bo qua</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>11/13</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>LOI</t>
         </is>
       </c>
     </row>

</xml_diff>